<commit_message>
docs: standardize Black Box and White Box sheets to identical 9-column college template
</commit_message>
<xml_diff>
--- a/test/A1_B4_52_PRANAV_RATHI_BLACK_BOX.xlsx
+++ b/test/A1_B4_52_PRANAV_RATHI_BLACK_BOX.xlsx
@@ -572,7 +572,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>30-09-2026</t>
+          <t>30 09 2026</t>
         </is>
       </c>
     </row>
@@ -636,7 +636,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="36" customHeight="1">
+    <row r="9" ht="34" customHeight="1">
       <c r="A9" s="6" t="n">
         <v>1</v>
       </c>
@@ -685,7 +685,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="36" customHeight="1">
+    <row r="10" ht="34" customHeight="1">
       <c r="A10" s="6" t="n">
         <v>2</v>
       </c>
@@ -733,7 +733,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="36" customHeight="1">
+    <row r="11" ht="34" customHeight="1">
       <c r="A11" s="6" t="n">
         <v>3</v>
       </c>
@@ -749,9 +749,9 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Product: Laptop
-Product ID: WMS-101
-Qty: 25</t>
+          <t>Product: Keyboard
+Product ID: P001
+Qty: 20</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -783,7 +783,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="36" customHeight="1">
+    <row r="12" ht="34" customHeight="1">
       <c r="A12" s="6" t="n">
         <v>4</v>
       </c>
@@ -800,7 +800,7 @@
       <c r="D12" s="7" t="inlineStr">
         <is>
           <t>Product Name: blank
-Product ID: WMS-102</t>
+Product ID: P002</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
@@ -831,7 +831,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="36" customHeight="1">
+    <row r="13" ht="34" customHeight="1">
       <c r="A13" s="6" t="n">
         <v>5</v>
       </c>
@@ -842,91 +842,91 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
+          <t>Add product with existing ID</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Product ID: P001</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>P001 already exists</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>1. Open Add Product
+2. Enter Product ID P001
+3. Click Save</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>Duplicate Product ID should not be accepted.</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Duplicate Product ID message was shown.</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>TC_006</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
           <t>Add product with empty Product ID</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D14" s="7" t="inlineStr">
         <is>
           <t>Product ID: blank
 Name: iPhone 16 Pro</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="E14" s="7" t="inlineStr">
         <is>
           <t>Add Product page is open</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr">
+      <c r="F14" s="7" t="inlineStr">
         <is>
           <t>1. Leave Product ID empty
 2. Enter name
 3. Click Save</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr">
+      <c r="G14" s="7" t="inlineStr">
         <is>
           <t>System should ask for Product ID.</t>
         </is>
       </c>
-      <c r="H13" s="7" t="inlineStr">
+      <c r="H14" s="7" t="inlineStr">
         <is>
           <t>Product ID required message was shown.</t>
         </is>
       </c>
-      <c r="I13" s="8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="36" customHeight="1">
-      <c r="A14" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>TC_006</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>Add product with duplicate ID</t>
-        </is>
-      </c>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t>Product ID: WMS-101
-(Already exists)</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="inlineStr">
-        <is>
-          <t>WMS-101 already exists</t>
-        </is>
-      </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>1. Enter existing Product ID WMS-101
-2. Click Save</t>
-        </is>
-      </c>
-      <c r="G14" s="7" t="inlineStr">
-        <is>
-          <t>Duplicate Product ID should not be accepted.</t>
-        </is>
-      </c>
-      <c r="H14" s="7" t="inlineStr">
-        <is>
-          <t>Duplicate Product ID message was shown.</t>
-        </is>
-      </c>
       <c r="I14" s="8" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="36" customHeight="1">
+    <row r="15" ht="34" customHeight="1">
       <c r="A15" s="6" t="n">
         <v>7</v>
       </c>
@@ -973,7 +973,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="36" customHeight="1">
+    <row r="16" ht="34" customHeight="1">
       <c r="A16" s="6" t="n">
         <v>8</v>
       </c>
@@ -1020,7 +1020,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="36" customHeight="1">
+    <row r="17" ht="34" customHeight="1">
       <c r="A17" s="6" t="n">
         <v>9</v>
       </c>
@@ -1067,7 +1067,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="36" customHeight="1">
+    <row r="18" ht="34" customHeight="1">
       <c r="A18" s="6" t="n">
         <v>10</v>
       </c>
@@ -1114,7 +1114,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="36" customHeight="1">
+    <row r="19" ht="34" customHeight="1">
       <c r="A19" s="6" t="n">
         <v>11</v>
       </c>
@@ -1160,7 +1160,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="36" customHeight="1">
+    <row r="20" ht="34" customHeight="1">
       <c r="A20" s="6" t="n">
         <v>12</v>
       </c>
@@ -1206,7 +1206,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="36" customHeight="1">
+    <row r="21" ht="34" customHeight="1">
       <c r="A21" s="6" t="n">
         <v>13</v>
       </c>
@@ -1251,7 +1251,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="36" customHeight="1">
+    <row r="22" ht="34" customHeight="1">
       <c r="A22" s="6" t="n">
         <v>14</v>
       </c>
@@ -1297,7 +1297,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="36" customHeight="1">
+    <row r="23" ht="34" customHeight="1">
       <c r="A23" s="6" t="n">
         <v>15</v>
       </c>
@@ -1342,7 +1342,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="36" customHeight="1">
+    <row r="24" ht="34" customHeight="1">
       <c r="A24" s="6" t="n">
         <v>16</v>
       </c>
@@ -1390,7 +1390,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="36" customHeight="1">
+    <row r="25" ht="34" customHeight="1">
       <c r="A25" s="6" t="n">
         <v>17</v>
       </c>
@@ -1436,7 +1436,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="36" customHeight="1">
+    <row r="26" ht="34" customHeight="1">
       <c r="A26" s="6" t="n">
         <v>18</v>
       </c>
@@ -1484,7 +1484,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="36" customHeight="1">
+    <row r="27" ht="34" customHeight="1">
       <c r="A27" s="6" t="n">
         <v>19</v>
       </c>
@@ -1531,7 +1531,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="36" customHeight="1">
+    <row r="28" ht="34" customHeight="1">
       <c r="A28" s="6" t="n">
         <v>20</v>
       </c>
@@ -1577,7 +1577,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="36" customHeight="1">
+    <row r="29" ht="34" customHeight="1">
       <c r="A29" s="6" t="n">
         <v>21</v>
       </c>
@@ -1623,7 +1623,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="36" customHeight="1">
+    <row r="30" ht="34" customHeight="1">
       <c r="A30" s="6" t="n">
         <v>22</v>
       </c>
@@ -1671,7 +1671,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="36" customHeight="1">
+    <row r="31" ht="34" customHeight="1">
       <c r="A31" s="6" t="n">
         <v>23</v>
       </c>
@@ -1718,7 +1718,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="36" customHeight="1">
+    <row r="32" ht="34" customHeight="1">
       <c r="A32" s="6" t="n">
         <v>24</v>
       </c>
@@ -1765,7 +1765,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="36" customHeight="1">
+    <row r="33" ht="34" customHeight="1">
       <c r="A33" s="6" t="n">
         <v>25</v>
       </c>
@@ -1811,7 +1811,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="36" customHeight="1">
+    <row r="34" ht="34" customHeight="1">
       <c r="A34" s="6" t="n">
         <v>26</v>
       </c>
@@ -1857,7 +1857,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="36" customHeight="1">
+    <row r="35" ht="34" customHeight="1">
       <c r="A35" s="6" t="n">
         <v>27</v>
       </c>
@@ -1902,7 +1902,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="36" customHeight="1">
+    <row r="36" ht="34" customHeight="1">
       <c r="A36" s="6" t="n">
         <v>28</v>
       </c>
@@ -1947,7 +1947,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="36" customHeight="1">
+    <row r="37" ht="34" customHeight="1">
       <c r="A37" s="6" t="n">
         <v>29</v>
       </c>
@@ -1992,7 +1992,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="36" customHeight="1">
+    <row r="38" ht="34" customHeight="1">
       <c r="A38" s="6" t="n">
         <v>30</v>
       </c>

</xml_diff>